<commit_message>
codex: generate LEAP pair registry from model rows
Builds the review-only LEAP structural key-pair registry from all current economy export templates and the demand/power detailed-row sheets. Adds source fingerprint refresh, provenance, structural coverage QA, refreshed prototype workbooks, and records the deferred workbook relocation.\n\nVerification: 39 focused tests passed; generated master loaded with 2,426 active relationships, zero incomplete rows, and 4,852 Stage 1 rows. Canonical master unchanged.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis_prototype.xlsx
+++ b/config/outlook_mappings_single_axis_prototype.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R981edea852d1472f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Ra86ecd88087a43d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R3a1e67b5d65b4f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="Rd6c7029ad8734410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R1071416c99d040d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rdc23ecef3a174468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rd241d7f9a22448c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R248a14f82b344076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R90d6419bd5e146c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R1bc02263090d4a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R8b2142a806ae4316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R049b75b243eb42f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rca94347e6e7d4825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rd5f225a57db74db9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>